<commit_message>
Update ImportTemplate.xlsx with new data structure
</commit_message>
<xml_diff>
--- a/rsc/templates/ImportTemplate.xlsx
+++ b/rsc/templates/ImportTemplate.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\rsc\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06D2F8B3-69E5-4B5F-BA07-30F6DB379C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC83F5C5-6E39-43F6-A2BF-2E06F7CECF3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4920" yWindow="5535" windowWidth="33480" windowHeight="17565" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="16440" yWindow="7575" windowWidth="33480" windowHeight="17565" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Dataset" sheetId="1" r:id="rId1"/>
+    <sheet name="Dataset2" sheetId="1" r:id="rId1"/>
     <sheet name="Config" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
@@ -2062,7 +2062,7 @@
         <v>98</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>58</v>
@@ -2677,26 +2677,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -2925,26 +2905,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2961,4 +2942,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>